<commit_message>
Fix quote template layout clipping
Merge label cells (A:B) and value cells (C:E) for the case-info block,
move grand total and validity date to two-row merged F:G blocks, and
merge the issuer/invoice-number lines so labels no longer clip or overlap.
Recalc verified: 40 formulas, 0 errors, sample total 976,100 JPY.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCH9AqPSyAXQdBeuY9N4qp
</commit_message>
<xml_diff>
--- a/templates/見積書テンプレ_v1.xlsx
+++ b/templates/見積書テンプレ_v1.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="59">
   <si>
     <t xml:space="preserve">御 見 積 書</t>
   </si>
@@ -210,7 +210,28 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">インボイス登録番号</t>
+      <t xml:space="preserve">インボイス登録番号 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">T</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">担当</t>
     </r>
     <r>
       <rPr>
@@ -224,37 +245,278 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">担当</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">:</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">件名</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">御見積合計</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">税込</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">ご利用期間</t>
   </si>
   <si>
+    <t xml:space="preserve">ご利用人数</t>
+  </si>
+  <si>
+    <t xml:space="preserve">お支払方法</t>
+  </si>
+  <si>
+    <t xml:space="preserve">見積有効期限</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">項目</t>
+  </si>
+  <si>
+    <t xml:space="preserve">内容</t>
+  </si>
+  <si>
+    <t xml:space="preserve">単価</t>
+  </si>
+  <si>
+    <t xml:space="preserve">数量</t>
+  </si>
+  <si>
+    <t xml:space="preserve">単位</t>
+  </si>
+  <si>
+    <t xml:space="preserve">金額</t>
+  </si>
+  <si>
+    <t xml:space="preserve">小計</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">サービス料</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10%)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">消費税</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10%)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">※入湯税</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=150</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">宿泊人数</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">泊数</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">手入力</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">入湯税</t>
+  </si>
+  <si>
+    <t xml:space="preserve">※値引きはマイナスで入力</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">お値引き</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">マイナス入力</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
@@ -264,7 +526,7 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -275,7 +537,7 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
@@ -285,7 +547,7 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -295,151 +557,79 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">ご利用人数</t>
-  </si>
-  <si>
-    <t xml:space="preserve">お支払方法</t>
-  </si>
-  <si>
-    <t xml:space="preserve">見積有効期限</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">項目</t>
-  </si>
-  <si>
-    <t xml:space="preserve">内容</t>
-  </si>
-  <si>
-    <t xml:space="preserve">単価</t>
-  </si>
-  <si>
-    <t xml:space="preserve">数量</t>
-  </si>
-  <si>
-    <t xml:space="preserve">単位</t>
-  </si>
-  <si>
-    <t xml:space="preserve">金額</t>
-  </si>
-  <si>
-    <t xml:space="preserve">小計</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">サービス料</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(10%)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">消費税</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(10%)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">※入湯税</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=150</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">円</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">×</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">宿泊人数</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">×</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">泊数</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
+    <t xml:space="preserve">備考</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【使い方】黄色セル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">入力欄 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">白セル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">自動計算</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
         <charset val="1"/>
@@ -449,42 +639,192 @@
     <r>
       <rPr>
         <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">手入力</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">触らない</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">)</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">入湯税</t>
-  </si>
-  <si>
-    <t xml:space="preserve">※値引きはマイナスで入力</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">お値引き</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。金額列・小計・税・合計は数式です。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">サービス料率・消費税率を変える場合は該当行の数式内の </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を修正。ロゴは【ロゴ】枠に画像を挿入。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Q-2026-0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026/7/17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0815TANA01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">田中産業株式会社  御中</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ご担当</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">田中 一郎 様</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">インボイス登録番号 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">T0000000000000</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">清水 祥太郎</t>
+  </si>
+  <si>
+    <t xml:space="preserve">田中産業株式会社様 ご宴会・ご宿泊</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">月</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -494,16 +834,16 @@
     </r>
     <r>
       <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">マイナス入力</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">土</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -511,22 +851,37 @@
       </rPr>
       <t xml:space="preserve">)</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">御見積合計</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -536,18 +891,113 @@
     </r>
     <r>
       <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">税込</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">泊</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">大人</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -557,79 +1007,19 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">備考</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">【使い方】黄色セル</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">入力欄 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">白セル</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">自動計算</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">後日振込</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
         <charset val="1"/>
@@ -638,379 +1028,7 @@
     </r>
     <r>
       <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">触らない</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。金額列・小計・税・合計は数式です。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">サービス料率・消費税率を変える場合は該当行の数式内の </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">を修正。ロゴは【ロゴ】枠に画像を挿入。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Q-2026-0001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/7/17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0815TANA01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">田中産業株式会社  御中</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ご担当</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">田中 一郎 様</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">T0000000000000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">清水 祥太郎</t>
-  </si>
-  <si>
-    <t xml:space="preserve">田中産業株式会社様 ご宴会・ご宿泊</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2026</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">年</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">月</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">土</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">〜</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">16</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) 1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">泊</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">名</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">大人</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">名</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">後日振込</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
+        <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
@@ -1019,7 +1037,7 @@
     </r>
     <r>
       <rPr>
-        <sz val="9"/>
+        <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -1029,7 +1047,7 @@
     </r>
     <r>
       <rPr>
-        <sz val="9"/>
+        <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
@@ -1038,7 +1056,7 @@
     </r>
     <r>
       <rPr>
-        <sz val="9"/>
+        <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -1607,7 +1625,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1644,19 +1662,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1668,30 +1682,34 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1732,10 +1750,6 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="166" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1757,10 +1771,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="23" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2099,87 +2109,99 @@
       <c r="F6" s="9" t="s">
         <v>8</v>
       </c>
+      <c r="G6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F7" s="10" t="s">
         <v>9</v>
       </c>
+      <c r="G7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F8" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="12"/>
+      <c r="G8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="14"/>
+      <c r="G9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-    </row>
-    <row r="11" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="B10" s="14"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="F11" s="17" t="s">
+      <c r="G10" s="16"/>
+    </row>
+    <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="18" t="n">
+      <c r="B11" s="14"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="17" t="n">
         <f aca="false">G36</f>
         <v>0</v>
       </c>
+      <c r="G11" s="17"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="F13" s="15" t="s">
+      <c r="B13" s="14"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="4"/>
+      <c r="G13" s="14"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G15" s="20" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2465,64 +2487,75 @@
       <c r="A36" s="26"/>
       <c r="B36" s="26"/>
       <c r="C36" s="26"/>
-      <c r="D36" s="31" t="s">
+      <c r="D36" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="32" t="n">
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="31" t="n">
         <f aca="false">G31+G32+G33+N(G34)+N(G35)</f>
         <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="s">
+      <c r="A38" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B38" s="33"/>
-      <c r="C38" s="33"/>
-      <c r="D38" s="33"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="33"/>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="33"/>
-      <c r="C39" s="33"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="33"/>
-      <c r="G39" s="33"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="33"/>
-      <c r="C40" s="33"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33"/>
-      <c r="G40" s="33"/>
+      <c r="B40" s="32"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="32"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="34" t="s">
+      <c r="A42" s="33" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="34" t="s">
+      <c r="A43" s="33" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="33">
     <mergeCell ref="B1:E2"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:G5"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="D31:F31"/>
     <mergeCell ref="A32:C32"/>
@@ -2598,12 +2631,12 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
       <c r="F4" s="6" t="s">
         <v>5</v>
       </c>
@@ -2629,101 +2662,111 @@
       <c r="F6" s="9" t="s">
         <v>8</v>
       </c>
+      <c r="G6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F7" s="10" t="s">
         <v>9</v>
       </c>
+      <c r="G7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F8" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="12" t="s">
         <v>41</v>
       </c>
+      <c r="G8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="36" t="s">
+      <c r="G9" s="35" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="14"/>
+      <c r="C10" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-    </row>
-    <row r="11" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="G10" s="16"/>
+    </row>
+    <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="14"/>
+      <c r="C11" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="F11" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="G11" s="18" t="n">
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="17" t="n">
         <f aca="false">G36</f>
         <v>976100</v>
       </c>
+      <c r="G11" s="17"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="14"/>
+      <c r="C12" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="38" t="s">
+      <c r="B13" s="14"/>
+      <c r="C13" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="F13" s="15" t="s">
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="14"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F14" s="18" t="s">
         <v>47</v>
       </c>
+      <c r="G14" s="18"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G15" s="20" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2731,7 +2774,7 @@
       <c r="A16" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="39" t="s">
+      <c r="B16" s="37" t="s">
         <v>48</v>
       </c>
       <c r="C16" s="22" t="s">
@@ -2743,7 +2786,7 @@
       <c r="E16" s="24" t="n">
         <v>40</v>
       </c>
-      <c r="F16" s="40" t="s">
+      <c r="F16" s="38" t="s">
         <v>50</v>
       </c>
       <c r="G16" s="25" t="n">
@@ -2755,10 +2798,10 @@
       <c r="A17" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="37" t="s">
         <v>52</v>
       </c>
       <c r="D17" s="23" t="n">
@@ -2767,7 +2810,7 @@
       <c r="E17" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="40" t="s">
+      <c r="F17" s="38" t="s">
         <v>53</v>
       </c>
       <c r="G17" s="25" t="n">
@@ -2779,10 +2822,10 @@
       <c r="A18" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="39" t="s">
+      <c r="C18" s="37" t="s">
         <v>54</v>
       </c>
       <c r="D18" s="23" t="n">
@@ -2791,7 +2834,7 @@
       <c r="E18" s="24" t="n">
         <v>40</v>
       </c>
-      <c r="F18" s="40" t="s">
+      <c r="F18" s="38" t="s">
         <v>50</v>
       </c>
       <c r="G18" s="25" t="n">
@@ -2803,10 +2846,10 @@
       <c r="A19" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="39" t="s">
+      <c r="C19" s="37" t="s">
         <v>56</v>
       </c>
       <c r="D19" s="23" t="n">
@@ -2815,7 +2858,7 @@
       <c r="E19" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="40" t="s">
+      <c r="F19" s="38" t="s">
         <v>57</v>
       </c>
       <c r="G19" s="25" t="n">
@@ -2827,11 +2870,11 @@
       <c r="A20" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
       <c r="D20" s="23"/>
       <c r="E20" s="24"/>
-      <c r="F20" s="40"/>
+      <c r="F20" s="38"/>
       <c r="G20" s="25" t="str">
         <f aca="false">IF(COUNT(D20,E20)&lt;2,"",D20*E20)</f>
         <v/>
@@ -2841,11 +2884,11 @@
       <c r="A21" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B21" s="39"/>
-      <c r="C21" s="39"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
       <c r="D21" s="23"/>
       <c r="E21" s="24"/>
-      <c r="F21" s="40"/>
+      <c r="F21" s="38"/>
       <c r="G21" s="25" t="str">
         <f aca="false">IF(COUNT(D21,E21)&lt;2,"",D21*E21)</f>
         <v/>
@@ -2855,11 +2898,11 @@
       <c r="A22" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="B22" s="39"/>
-      <c r="C22" s="39"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
       <c r="D22" s="23"/>
       <c r="E22" s="24"/>
-      <c r="F22" s="40"/>
+      <c r="F22" s="38"/>
       <c r="G22" s="25" t="str">
         <f aca="false">IF(COUNT(D22,E22)&lt;2,"",D22*E22)</f>
         <v/>
@@ -2869,11 +2912,11 @@
       <c r="A23" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B23" s="39"/>
-      <c r="C23" s="39"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
       <c r="D23" s="23"/>
       <c r="E23" s="24"/>
-      <c r="F23" s="40"/>
+      <c r="F23" s="38"/>
       <c r="G23" s="25" t="str">
         <f aca="false">IF(COUNT(D23,E23)&lt;2,"",D23*E23)</f>
         <v/>
@@ -2883,11 +2926,11 @@
       <c r="A24" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="B24" s="39"/>
-      <c r="C24" s="39"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
       <c r="D24" s="23"/>
       <c r="E24" s="24"/>
-      <c r="F24" s="40"/>
+      <c r="F24" s="38"/>
       <c r="G24" s="25" t="str">
         <f aca="false">IF(COUNT(D24,E24)&lt;2,"",D24*E24)</f>
         <v/>
@@ -2897,11 +2940,11 @@
       <c r="A25" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="B25" s="39"/>
-      <c r="C25" s="39"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
       <c r="D25" s="23"/>
       <c r="E25" s="24"/>
-      <c r="F25" s="40"/>
+      <c r="F25" s="38"/>
       <c r="G25" s="25" t="str">
         <f aca="false">IF(COUNT(D25,E25)&lt;2,"",D25*E25)</f>
         <v/>
@@ -2911,11 +2954,11 @@
       <c r="A26" s="21" t="n">
         <v>11</v>
       </c>
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
       <c r="D26" s="23"/>
       <c r="E26" s="24"/>
-      <c r="F26" s="40"/>
+      <c r="F26" s="38"/>
       <c r="G26" s="25" t="str">
         <f aca="false">IF(COUNT(D26,E26)&lt;2,"",D26*E26)</f>
         <v/>
@@ -2925,11 +2968,11 @@
       <c r="A27" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="B27" s="39"/>
-      <c r="C27" s="39"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
       <c r="D27" s="23"/>
       <c r="E27" s="24"/>
-      <c r="F27" s="40"/>
+      <c r="F27" s="38"/>
       <c r="G27" s="25" t="str">
         <f aca="false">IF(COUNT(D27,E27)&lt;2,"",D27*E27)</f>
         <v/>
@@ -2939,11 +2982,11 @@
       <c r="A28" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="B28" s="39"/>
-      <c r="C28" s="39"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
       <c r="D28" s="23"/>
       <c r="E28" s="24"/>
-      <c r="F28" s="40"/>
+      <c r="F28" s="38"/>
       <c r="G28" s="25" t="str">
         <f aca="false">IF(COUNT(D28,E28)&lt;2,"",D28*E28)</f>
         <v/>
@@ -2953,11 +2996,11 @@
       <c r="A29" s="21" t="n">
         <v>14</v>
       </c>
-      <c r="B29" s="39"/>
-      <c r="C29" s="39"/>
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
       <c r="D29" s="23"/>
       <c r="E29" s="24"/>
-      <c r="F29" s="40"/>
+      <c r="F29" s="38"/>
       <c r="G29" s="25" t="str">
         <f aca="false">IF(COUNT(D29,E29)&lt;2,"",D29*E29)</f>
         <v/>
@@ -2967,11 +3010,11 @@
       <c r="A30" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39"/>
+      <c r="B30" s="37"/>
+      <c r="C30" s="37"/>
       <c r="D30" s="23"/>
       <c r="E30" s="24"/>
-      <c r="F30" s="40"/>
+      <c r="F30" s="38"/>
       <c r="G30" s="25" t="str">
         <f aca="false">IF(COUNT(D30,E30)&lt;2,"",D30*E30)</f>
         <v/>
@@ -3053,66 +3096,77 @@
       <c r="A36" s="26"/>
       <c r="B36" s="26"/>
       <c r="C36" s="26"/>
-      <c r="D36" s="31" t="s">
+      <c r="D36" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="32" t="n">
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="31" t="n">
         <f aca="false">G31+G32+G33+N(G34)+N(G35)</f>
         <v>976100</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="s">
+      <c r="A38" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B38" s="41" t="s">
+      <c r="B38" s="39" t="s">
         <v>58</v>
       </c>
-      <c r="C38" s="41"/>
-      <c r="D38" s="41"/>
-      <c r="E38" s="41"/>
-      <c r="F38" s="41"/>
-      <c r="G38" s="41"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="41"/>
-      <c r="C39" s="41"/>
-      <c r="D39" s="41"/>
-      <c r="E39" s="41"/>
-      <c r="F39" s="41"/>
-      <c r="G39" s="41"/>
+      <c r="B39" s="39"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="39"/>
+      <c r="G39" s="39"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="41"/>
-      <c r="C40" s="41"/>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="41"/>
-      <c r="G40" s="41"/>
+      <c r="B40" s="39"/>
+      <c r="C40" s="39"/>
+      <c r="D40" s="39"/>
+      <c r="E40" s="39"/>
+      <c r="F40" s="39"/>
+      <c r="G40" s="39"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="34" t="s">
+      <c r="A42" s="33" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="34" t="s">
+      <c r="A43" s="33" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="33">
     <mergeCell ref="B1:E2"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:G5"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="D31:F31"/>
     <mergeCell ref="A32:C32"/>

</xml_diff>

<commit_message>
Add company/group/tour name fields; hide empty fields in output
Split the addressee into three inputs (会社名/団体名/ツアー名, at least
one required) per Sho's real-case feedback. Record the rule that blank
fields are skipped in generated documents; the manual Excel template
notes row-hiding for unused name lines. Recalc verified, 0 errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCH9AqPSyAXQdBeuY9N4qp
</commit_message>
<xml_diff>
--- a/templates/見積書テンプレ_v1.xlsx
+++ b/templates/見積書テンプレ_v1.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="64">
   <si>
     <t xml:space="preserve">御 見 積 書</t>
   </si>
@@ -58,7 +58,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">団体名</t>
+      <t xml:space="preserve">会社名</t>
     </r>
     <r>
       <rPr>
@@ -88,6 +88,102 @@
   <si>
     <r>
       <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">団体名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ツアー名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ホテル名</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
         <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
@@ -135,14 +231,100 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">住所・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TEL)</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">下記のとおりお見積り申し上げます。</t>
   </si>
   <si>
     <r>
       <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">インボイス登録番号 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">T</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">担当</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">:</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">件名</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
         <b val="true"/>
         <sz val="10"/>
         <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">御見積合計</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
         <charset val="1"/>
@@ -157,7 +339,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">ホテル名</t>
+      <t xml:space="preserve">税込</t>
     </r>
     <r>
       <rPr>
@@ -172,10 +354,154 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
+    <t xml:space="preserve">ご利用期間</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ご利用人数</t>
+  </si>
+  <si>
+    <t xml:space="preserve">お支払方法</t>
+  </si>
+  <si>
+    <t xml:space="preserve">見積有効期限</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">項目</t>
+  </si>
+  <si>
+    <t xml:space="preserve">内容</t>
+  </si>
+  <si>
+    <t xml:space="preserve">単価</t>
+  </si>
+  <si>
+    <t xml:space="preserve">数量</t>
+  </si>
+  <si>
+    <t xml:space="preserve">単位</t>
+  </si>
+  <si>
+    <t xml:space="preserve">金額</t>
+  </si>
+  <si>
+    <t xml:space="preserve">小計</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">サービス料</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10%)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">消費税</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10%)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">※入湯税</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=150</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">宿泊人数</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">泊数</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
         <charset val="1"/>
@@ -185,73 +511,74 @@
     <r>
       <rPr>
         <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">住所・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">TEL)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">インボイス登録番号 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">T</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">担当</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">:</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">件名</t>
+        <color rgb="FF888888"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">手入力</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF888888"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">入湯税</t>
+  </si>
+  <si>
+    <t xml:space="preserve">※値引きはマイナスで入力</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">お値引き</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">マイナス入力</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
@@ -261,7 +588,7 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -272,7 +599,7 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
@@ -282,7 +609,7 @@
     <r>
       <rPr>
         <b val="true"/>
-        <sz val="10"/>
+        <sz val="9"/>
         <color rgb="FF000000"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
@@ -292,154 +619,79 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">ご利用期間</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ご利用人数</t>
-  </si>
-  <si>
-    <t xml:space="preserve">お支払方法</t>
-  </si>
-  <si>
-    <t xml:space="preserve">見積有効期限</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">項目</t>
-  </si>
-  <si>
-    <t xml:space="preserve">内容</t>
-  </si>
-  <si>
-    <t xml:space="preserve">単価</t>
-  </si>
-  <si>
-    <t xml:space="preserve">数量</t>
-  </si>
-  <si>
-    <t xml:space="preserve">単位</t>
-  </si>
-  <si>
-    <t xml:space="preserve">金額</t>
-  </si>
-  <si>
-    <t xml:space="preserve">小計</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">サービス料</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(10%)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">消費税</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(10%)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">※入湯税</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=150</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">円</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">×</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">宿泊人数</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">×</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">泊数</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
+    <t xml:space="preserve">備考</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【使い方】黄色セル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">入力欄 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">白セル</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">自動計算</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
         <charset val="1"/>
@@ -449,117 +701,158 @@
     <r>
       <rPr>
         <sz val="8"/>
-        <color rgb="FF888888"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">手入力</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF888888"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">触らない</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">)</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">入湯税</t>
-  </si>
-  <si>
-    <t xml:space="preserve">※値引きはマイナスで入力</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">お値引き</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">マイナス入力</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。金額列・小計・税・合計は数式です。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">サービス料率・消費税率を変える場合は該当行の数式内の </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を修正。ロゴは【ロゴ】枠に画像を挿入。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">会社名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">団体名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ツアー名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">行目</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF666666"/>
         <rFont val="Yu Gothic"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">)</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">御見積合計</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">税込</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">備考</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="8"/>
@@ -567,132 +860,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【使い方】黄色セル</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">入力欄 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">白セル</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">自動計算</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">触らない</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。金額列・小計・税・合計は数式です。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">サービス料率・消費税率を変える場合は該当行の数式内の </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="Yu Gothic"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF666666"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">を修正。ロゴは【ロゴ】枠に画像を挿入。</t>
+      <t xml:space="preserve">で使わない行は、行番号を右クリック→「非表示」にしてから印刷すると空欄が出ません。</t>
     </r>
   </si>
   <si>
@@ -706,6 +874,30 @@
   </si>
   <si>
     <t xml:space="preserve">田中産業株式会社  御中</t>
+  </si>
+  <si>
+    <t xml:space="preserve">田中産業 親睦会ご一行様</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Yu Gothic"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年度 社員親睦旅行「妙高高原の旅」</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1428,6 +1620,19 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Yu Gothic"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1461,13 +1666,6 @@
       <color rgb="FF000000"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Yu Gothic"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -1518,12 +1716,6 @@
       <name val="Yu Gothic"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1625,7 +1817,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1654,27 +1846,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1682,19 +1878,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1702,11 +1898,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1730,7 +1926,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1742,7 +1938,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1750,7 +1946,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1758,7 +1954,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1766,11 +1962,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2038,7 +2238,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.5"/>
@@ -2100,449 +2300,468 @@
       <c r="G5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="F6" s="9" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="F6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="9"/>
+      <c r="G6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
       <c r="F7" s="10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F8" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="11"/>
+      <c r="A8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="F8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F9" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="13"/>
+      <c r="F9" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="16"/>
+      <c r="A10" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="15"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="17"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="17" t="n">
+      <c r="A11" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="15"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="18" t="n">
         <f aca="false">G36</f>
         <v>0</v>
       </c>
-      <c r="G11" s="17"/>
+      <c r="G11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
+      <c r="A12" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="14"/>
+      <c r="A13" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="20" t="s">
+      <c r="A15" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="B15" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="C15" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="20" t="s">
+      <c r="D15" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="E15" s="21" t="s">
         <v>24</v>
       </c>
+      <c r="F15" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="24"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="25"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="25" t="str">
+      <c r="G16" s="26" t="str">
         <f aca="false">IF(COUNT(D16,E16)&lt;2,"",D16*E16)</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="24"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="25"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="25" t="str">
+      <c r="G17" s="26" t="str">
         <f aca="false">IF(COUNT(D17,E17)&lt;2,"",D17*E17)</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="24"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="25"/>
       <c r="F18" s="3"/>
-      <c r="G18" s="25" t="str">
+      <c r="G18" s="26" t="str">
         <f aca="false">IF(COUNT(D18,E18)&lt;2,"",D18*E18)</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="24"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="25"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="25" t="str">
+      <c r="G19" s="26" t="str">
         <f aca="false">IF(COUNT(D19,E19)&lt;2,"",D19*E19)</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="24"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="25"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="25" t="str">
+      <c r="G20" s="26" t="str">
         <f aca="false">IF(COUNT(D20,E20)&lt;2,"",D20*E20)</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="24"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="25"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="25" t="str">
+      <c r="G21" s="26" t="str">
         <f aca="false">IF(COUNT(D21,E21)&lt;2,"",D21*E21)</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="n">
+      <c r="A22" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="24"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="25"/>
       <c r="F22" s="3"/>
-      <c r="G22" s="25" t="str">
+      <c r="G22" s="26" t="str">
         <f aca="false">IF(COUNT(D22,E22)&lt;2,"",D22*E22)</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="n">
+      <c r="A23" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="24"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="25"/>
       <c r="F23" s="3"/>
-      <c r="G23" s="25" t="str">
+      <c r="G23" s="26" t="str">
         <f aca="false">IF(COUNT(D23,E23)&lt;2,"",D23*E23)</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="n">
+      <c r="A24" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="24"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="25"/>
       <c r="F24" s="3"/>
-      <c r="G24" s="25" t="str">
+      <c r="G24" s="26" t="str">
         <f aca="false">IF(COUNT(D24,E24)&lt;2,"",D24*E24)</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="n">
+      <c r="A25" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="24"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="25"/>
       <c r="F25" s="3"/>
-      <c r="G25" s="25" t="str">
+      <c r="G25" s="26" t="str">
         <f aca="false">IF(COUNT(D25,E25)&lt;2,"",D25*E25)</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="n">
+      <c r="A26" s="22" t="n">
         <v>11</v>
       </c>
-      <c r="B26" s="22"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="24"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
       <c r="F26" s="3"/>
-      <c r="G26" s="25" t="str">
+      <c r="G26" s="26" t="str">
         <f aca="false">IF(COUNT(D26,E26)&lt;2,"",D26*E26)</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="n">
+      <c r="A27" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="24"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="3"/>
-      <c r="G27" s="25" t="str">
+      <c r="G27" s="26" t="str">
         <f aca="false">IF(COUNT(D27,E27)&lt;2,"",D27*E27)</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="n">
+      <c r="A28" s="22" t="n">
         <v>13</v>
       </c>
-      <c r="B28" s="22"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="24"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="25"/>
       <c r="F28" s="3"/>
-      <c r="G28" s="25" t="str">
+      <c r="G28" s="26" t="str">
         <f aca="false">IF(COUNT(D28,E28)&lt;2,"",D28*E28)</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="n">
+      <c r="A29" s="22" t="n">
         <v>14</v>
       </c>
-      <c r="B29" s="22"/>
-      <c r="C29" s="22"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="24"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="3"/>
-      <c r="G29" s="25" t="str">
+      <c r="G29" s="26" t="str">
         <f aca="false">IF(COUNT(D29,E29)&lt;2,"",D29*E29)</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="n">
+      <c r="A30" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="24"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="25"/>
       <c r="F30" s="3"/>
-      <c r="G30" s="25" t="str">
+      <c r="G30" s="26" t="str">
         <f aca="false">IF(COUNT(D30,E30)&lt;2,"",D30*E30)</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="28" t="n">
+      <c r="A31" s="27"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="29" t="n">
         <f aca="false">SUM(G16:G30)</f>
         <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="26"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="28" t="n">
+      <c r="A32" s="27"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="29" t="n">
         <f aca="false">ROUND(G31*0.1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="26"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="28" t="n">
+      <c r="A33" s="27"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="29" t="n">
         <f aca="false">ROUND((G31+G32)*0.1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" s="29"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="30"/>
+      <c r="A34" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="31"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" s="29"/>
-      <c r="C35" s="29"/>
-      <c r="D35" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="30"/>
+      <c r="A35" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="30"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="31"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="31" t="n">
+      <c r="A36" s="27"/>
+      <c r="B36" s="27"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="32" t="n">
         <f aca="false">G31+G32+G33+N(G34)+N(G35)</f>
         <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
+      <c r="A38" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" s="33"/>
+      <c r="C38" s="33"/>
+      <c r="D38" s="33"/>
+      <c r="E38" s="33"/>
+      <c r="F38" s="33"/>
+      <c r="G38" s="33"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
+      <c r="B39" s="33"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="33"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="33" t="s">
-        <v>34</v>
+      <c r="A42" s="34" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="33" t="s">
-        <v>35</v>
+      <c r="A43" s="34" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="34" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="35">
     <mergeCell ref="B1:E2"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:G5"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="F6:G6"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="A8:D8"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="C10:E10"/>
@@ -2585,7 +2804,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.5"/>
@@ -2607,7 +2826,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2619,7 +2838,7 @@
         <v>2</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2627,533 +2846,552 @@
         <v>3</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
+      <c r="A4" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
       <c r="F4" s="6" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
+      <c r="A5" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="F6" s="9" t="s">
+      <c r="A6" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="F6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="9"/>
+      <c r="G6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
       <c r="F7" s="10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F8" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="G8" s="11"/>
+      <c r="A8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="F8" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F9" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="35" t="s">
-        <v>42</v>
+      <c r="F9" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="37" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="36" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="16"/>
+      <c r="A10" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="15"/>
+      <c r="C10" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="17"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="17" t="n">
+      <c r="A11" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="15"/>
+      <c r="C11" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="18" t="n">
         <f aca="false">G36</f>
         <v>976100</v>
       </c>
-      <c r="G11" s="17"/>
+      <c r="G11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
+      <c r="A12" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="14"/>
+      <c r="A13" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F14" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="G14" s="18"/>
+      <c r="F14" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="19"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="20" t="s">
+      <c r="A15" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="B15" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="C15" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="20" t="s">
+      <c r="D15" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="E15" s="21" t="s">
         <v>24</v>
       </c>
+      <c r="F15" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="D16" s="23" t="n">
+      <c r="B16" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="24" t="n">
         <v>15000</v>
       </c>
-      <c r="E16" s="24" t="n">
+      <c r="E16" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="F16" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="G16" s="25" t="n">
+      <c r="F16" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" s="26" t="n">
         <f aca="false">IF(COUNT(D16,E16)&lt;2,"",D16*E16)</f>
         <v>600000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="37" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="37" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="23" t="n">
+      <c r="B17" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="39" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="24" t="n">
         <v>50000</v>
       </c>
-      <c r="E17" s="24" t="n">
+      <c r="E17" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="G17" s="25" t="n">
+      <c r="F17" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="G17" s="26" t="n">
         <f aca="false">IF(COUNT(D17,E17)&lt;2,"",D17*E17)</f>
         <v>50000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="37" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="37" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="23" t="n">
+      <c r="B18" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="24" t="n">
         <v>2500</v>
       </c>
-      <c r="E18" s="24" t="n">
+      <c r="E18" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="F18" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="G18" s="25" t="n">
+      <c r="F18" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="G18" s="26" t="n">
         <f aca="false">IF(COUNT(D18,E18)&lt;2,"",D18*E18)</f>
         <v>100000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B19" s="37" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="37" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" s="23" t="n">
+      <c r="B19" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="39" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="24" t="n">
         <v>30000</v>
       </c>
-      <c r="E19" s="24" t="n">
+      <c r="E19" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="38" t="s">
-        <v>57</v>
-      </c>
-      <c r="G19" s="25" t="n">
+      <c r="F19" s="40" t="s">
+        <v>62</v>
+      </c>
+      <c r="G19" s="26" t="n">
         <f aca="false">IF(COUNT(D19,E19)&lt;2,"",D19*E19)</f>
         <v>60000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="25" t="str">
+      <c r="B20" s="39"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="26" t="str">
         <f aca="false">IF(COUNT(D20,E20)&lt;2,"",D20*E20)</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="25" t="str">
+      <c r="B21" s="39"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="26" t="str">
         <f aca="false">IF(COUNT(D21,E21)&lt;2,"",D21*E21)</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="n">
+      <c r="A22" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="25" t="str">
+      <c r="B22" s="39"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="26" t="str">
         <f aca="false">IF(COUNT(D22,E22)&lt;2,"",D22*E22)</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="n">
+      <c r="A23" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="B23" s="37"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="25" t="str">
+      <c r="B23" s="39"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="26" t="str">
         <f aca="false">IF(COUNT(D23,E23)&lt;2,"",D23*E23)</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="n">
+      <c r="A24" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="B24" s="37"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="25" t="str">
+      <c r="B24" s="39"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="26" t="str">
         <f aca="false">IF(COUNT(D24,E24)&lt;2,"",D24*E24)</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="n">
+      <c r="A25" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="B25" s="37"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="25" t="str">
+      <c r="B25" s="39"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="26" t="str">
         <f aca="false">IF(COUNT(D25,E25)&lt;2,"",D25*E25)</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="n">
+      <c r="A26" s="22" t="n">
         <v>11</v>
       </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="25" t="str">
+      <c r="B26" s="39"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="26" t="str">
         <f aca="false">IF(COUNT(D26,E26)&lt;2,"",D26*E26)</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="n">
+      <c r="A27" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="25" t="str">
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="26" t="str">
         <f aca="false">IF(COUNT(D27,E27)&lt;2,"",D27*E27)</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="n">
+      <c r="A28" s="22" t="n">
         <v>13</v>
       </c>
-      <c r="B28" s="37"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="38"/>
-      <c r="G28" s="25" t="str">
+      <c r="B28" s="39"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="26" t="str">
         <f aca="false">IF(COUNT(D28,E28)&lt;2,"",D28*E28)</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="n">
+      <c r="A29" s="22" t="n">
         <v>14</v>
       </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="38"/>
-      <c r="G29" s="25" t="str">
+      <c r="B29" s="39"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="40"/>
+      <c r="G29" s="26" t="str">
         <f aca="false">IF(COUNT(D29,E29)&lt;2,"",D29*E29)</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="n">
+      <c r="A30" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="B30" s="37"/>
-      <c r="C30" s="37"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="38"/>
-      <c r="G30" s="25" t="str">
+      <c r="B30" s="39"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="26" t="str">
         <f aca="false">IF(COUNT(D30,E30)&lt;2,"",D30*E30)</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="28" t="n">
+      <c r="A31" s="27"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="29" t="n">
         <f aca="false">SUM(G16:G30)</f>
         <v>810000</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="26"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="28" t="n">
+      <c r="A32" s="27"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="29" t="n">
         <f aca="false">ROUND(G31*0.1,0)</f>
         <v>81000</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="26"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="28" t="n">
+      <c r="A33" s="27"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="29" t="n">
         <f aca="false">ROUND((G31+G32)*0.1,0)</f>
         <v>89100</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" s="29"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="30" t="n">
+      <c r="A34" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="31" t="n">
         <v>6000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="B35" s="29"/>
-      <c r="C35" s="29"/>
-      <c r="D35" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="30" t="n">
+      <c r="A35" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="30"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="31" t="n">
         <v>-10000</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="31" t="n">
+      <c r="A36" s="27"/>
+      <c r="B36" s="27"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="32" t="n">
         <f aca="false">G31+G32+G33+N(G34)+N(G35)</f>
         <v>976100</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="B38" s="39" t="s">
-        <v>58</v>
-      </c>
-      <c r="C38" s="39"/>
-      <c r="D38" s="39"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="39"/>
+      <c r="A38" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" s="41" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="41"/>
+      <c r="F38" s="41"/>
+      <c r="G38" s="41"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="39"/>
-      <c r="C39" s="39"/>
-      <c r="D39" s="39"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="39"/>
-      <c r="G39" s="39"/>
+      <c r="B39" s="41"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
+      <c r="F39" s="41"/>
+      <c r="G39" s="41"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="39"/>
-      <c r="C40" s="39"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="39"/>
-      <c r="G40" s="39"/>
+      <c r="B40" s="41"/>
+      <c r="C40" s="41"/>
+      <c r="D40" s="41"/>
+      <c r="E40" s="41"/>
+      <c r="F40" s="41"/>
+      <c r="G40" s="41"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="33" t="s">
-        <v>34</v>
+      <c r="A42" s="34" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="33" t="s">
-        <v>35</v>
+      <c r="A43" s="34" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="34" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="35">
     <mergeCell ref="B1:E2"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:G5"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="F6:G6"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="A8:D8"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="C10:E10"/>

</xml_diff>